<commit_message>
Buscador por presupuesto y lista de precios en la web; módulo de visitas guiadas; precios y documentos actualizados
- Web: "¿Qué lote me alcanza?" (cuota e inicial del cliente -> proyecto y plazo que encaja, con WhatsApp)
  e invitación a la lista de precios por WhatsApp (salida en computadora / lectura en celular, máx. 1 vez por semana).
- Herramienta: Visitas guiadas (agenda, confirmación y recordatorio por WhatsApp, .ics, asistencia), integradas en Hoy,
  Mis clientes, ranking, reporte gerencial, respaldo y consolidación del equipo. 14 módulos.
- Propuesta: Plan Comercial Integral S/ 25,900 (40/40/20: 10,360 / 10,360 / 5,180), Web S/ 12,000, Herramienta S/ 18,300;
  capturas nuevas con fotos reales y portada real. Presentación, contrato y manual actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SuYMBC9vy1hrR2C5YCk9db
</commit_message>
<xml_diff>
--- a/entregables/software/ejemplos-excel/ejemplo-reporte-gerencial.xlsx
+++ b/entregables/software/ejemplos-excel/ejemplo-reporte-gerencial.xlsx
@@ -10,7 +10,8 @@
     <sheet sheetId="4" name="Cobranza" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Clientes" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Asesores" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Inventario" state="visible" r:id="rId10"/>
+    <sheet sheetId="7" name="Visitas" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Inventario" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Resumen'!$10:$10</definedName>
@@ -19,14 +20,15 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Cobranza'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Clientes'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Asesores'!$7:$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Inventario'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Visitas'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Inventario'!$7:$7</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="172">
   <si>
     <t>REPORTE GERENCIAL COMERCIAL</t>
   </si>
@@ -95,6 +97,12 @@
   </si>
   <si>
     <t>Cobrado este mes</t>
+  </si>
+  <si>
+    <t>Visitas guiadas este mes</t>
+  </si>
+  <si>
+    <t>0 asistieron</t>
   </si>
   <si>
     <t>CLIENTES</t>
@@ -431,6 +439,9 @@
     <t>RANKING POR ASESOR (HISTÓRICO)</t>
   </si>
   <si>
+    <t>Visitas</t>
+  </si>
+  <si>
     <t>Proformas</t>
   </si>
   <si>
@@ -447,6 +458,18 @@
   </si>
   <si>
     <t>TOTAL EQUIPO</t>
+  </si>
+  <si>
+    <t>VISITAS GUIADAS</t>
+  </si>
+  <si>
+    <t>Hora</t>
+  </si>
+  <si>
+    <t>Punto de encuentro</t>
+  </si>
+  <si>
+    <t>Sin registros por ahora.</t>
   </si>
   <si>
     <t>INVENTARIO DE LOTES</t>
@@ -532,7 +555,7 @@
     <numFmt numFmtId="164" formatCode="&quot;S/&quot; #,##0"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -584,6 +607,12 @@
       <b/>
       <color rgb="FF0A3856"/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF6B7A86"/>
+      <sz val="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -690,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -798,6 +827,9 @@
     </xf>
     <xf numFmtId="1" fontId="8" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1090,6 +1122,50 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>96000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1809750" cy="371475"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1459,7 +1535,7 @@
     <tabColor rgb="FF0A3856"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -1639,172 +1715,184 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+    <row r="20" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B20"/>
-      <c r="C20"/>
-      <c r="D20"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="B20" s="14">
+        <v>0</v>
+      </c>
+      <c r="C20" s="15"/>
+      <c r="D20" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="11">
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="11">
         <v>1</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C22" s="12">
         <v>0</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="14">
+      <c r="D22" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="14">
         <v>3</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C23" s="15">
         <v>87000</v>
       </c>
-      <c r="D22" s="13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="D23" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="11">
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="11">
         <v>0</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C24" s="12">
         <v>0</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="14">
+      <c r="D24" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="14">
         <v>0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C25" s="15">
         <v>0</v>
       </c>
-      <c r="D24" s="13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="11">
+      <c r="D25" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="11">
         <v>1</v>
       </c>
-      <c r="C25" s="12">
+      <c r="C26" s="12">
         <v>29000</v>
       </c>
-      <c r="D25" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="14">
+      <c r="D26" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="14">
         <v>0</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C27" s="15">
         <v>0</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="17">
+      <c r="D27" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="17">
         <v>1</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="16" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+      <c r="C28" s="18"/>
+      <c r="D28" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="11">
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="11">
         <v>21</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C30" s="12">
         <v>609000</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="14">
+      <c r="D30" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="14">
         <v>0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C31" s="15">
         <v>0</v>
       </c>
-      <c r="D30" s="13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B31" s="11">
+      <c r="D31" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="11">
         <v>0</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C32" s="12">
         <v>0</v>
       </c>
-      <c r="D31" s="10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
+      <c r="D32" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B32" s="14">
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" s="14">
         <v>0</v>
       </c>
-      <c r="C32" s="15">
+      <c r="C33" s="15">
         <v>0</v>
       </c>
-      <c r="D32" s="13" t="s">
-        <v>37</v>
+      <c r="D33" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1815,8 +1903,8 @@
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A29:D29"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.2" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
@@ -1849,7 +1937,7 @@
     <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" ht="30" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -1879,163 +1967,163 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B8" s="19">
         <v>46320.5</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F8" s="12">
         <v>28000</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B9" s="20">
         <v>46320.5</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F9" s="15">
         <v>29000</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="19">
         <v>46320.5</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F10" s="12">
         <v>29000</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B11" s="20">
         <v>46320.5</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F11" s="15">
         <v>29000</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="19">
         <v>46320.5</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F12" s="12">
         <v>29000</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="21"/>
@@ -2085,7 +2173,7 @@
     <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" ht="30" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2115,51 +2203,51 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B8" s="19">
         <v>46320.5</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E8" s="12">
         <v>1500</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H8" s="19">
         <v>46327.5</v>
@@ -2167,7 +2255,7 @@
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -2217,7 +2305,7 @@
     <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" ht="30" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2247,28 +2335,28 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2276,22 +2364,22 @@
         <v>46327.5</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F8" s="27">
         <v>4300</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H8" s="28">
         <v>46320.5</v>
@@ -2302,22 +2390,22 @@
         <v>46336.5</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F9" s="15">
         <v>967</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H9" s="30"/>
     </row>
@@ -2326,22 +2414,22 @@
         <v>46366.5</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F10" s="12">
         <v>967</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H10" s="32"/>
     </row>
@@ -2350,22 +2438,22 @@
         <v>46397.5</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F11" s="15">
         <v>967</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H11" s="30"/>
     </row>
@@ -2374,22 +2462,22 @@
         <v>46428.5</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F12" s="12">
         <v>967</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H12" s="32"/>
     </row>
@@ -2398,22 +2486,22 @@
         <v>46456.5</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F13" s="15">
         <v>967</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H13" s="30"/>
     </row>
@@ -2422,22 +2510,22 @@
         <v>46487.5</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F14" s="12">
         <v>967</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H14" s="32"/>
     </row>
@@ -2446,22 +2534,22 @@
         <v>46517.5</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F15" s="15">
         <v>967</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H15" s="30"/>
     </row>
@@ -2470,22 +2558,22 @@
         <v>46548.5</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F16" s="12">
         <v>967</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H16" s="32"/>
     </row>
@@ -2494,22 +2582,22 @@
         <v>46578.5</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F17" s="15">
         <v>967</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H17" s="30"/>
     </row>
@@ -2518,22 +2606,22 @@
         <v>46609.5</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F18" s="12">
         <v>967</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H18" s="32"/>
     </row>
@@ -2542,22 +2630,22 @@
         <v>46640.5</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F19" s="15">
         <v>967</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H19" s="30"/>
     </row>
@@ -2566,22 +2654,22 @@
         <v>46670.5</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F20" s="12">
         <v>967</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H20" s="32"/>
     </row>
@@ -2590,22 +2678,22 @@
         <v>46701.5</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F21" s="15">
         <v>967</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H21" s="30"/>
     </row>
@@ -2614,22 +2702,22 @@
         <v>46731.5</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F22" s="12">
         <v>967</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H22" s="32"/>
     </row>
@@ -2638,22 +2726,22 @@
         <v>46762.5</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F23" s="15">
         <v>967</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H23" s="30"/>
     </row>
@@ -2662,22 +2750,22 @@
         <v>46793.5</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F24" s="12">
         <v>967</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H24" s="32"/>
     </row>
@@ -2686,22 +2774,22 @@
         <v>46822.5</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F25" s="15">
         <v>967</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H25" s="30"/>
     </row>
@@ -2710,22 +2798,22 @@
         <v>46853.5</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F26" s="12">
         <v>967</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H26" s="32"/>
     </row>
@@ -2734,22 +2822,22 @@
         <v>46883.5</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F27" s="15">
         <v>967</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H27" s="30"/>
     </row>
@@ -2758,22 +2846,22 @@
         <v>46914.5</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E28" s="31" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F28" s="12">
         <v>967</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H28" s="32"/>
     </row>
@@ -2782,22 +2870,22 @@
         <v>46944.5</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E29" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F29" s="15">
         <v>967</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H29" s="30"/>
     </row>
@@ -2806,22 +2894,22 @@
         <v>46975.5</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E30" s="31" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F30" s="12">
         <v>967</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H30" s="32"/>
     </row>
@@ -2830,22 +2918,22 @@
         <v>47006.5</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E31" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F31" s="15">
         <v>967</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H31" s="30"/>
     </row>
@@ -2854,28 +2942,28 @@
         <v>47036.5</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E32" s="31" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F32" s="12">
         <v>959</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H32" s="32"/>
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B33" s="21"/>
       <c r="C33" s="21"/>
@@ -2924,7 +3012,7 @@
     <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" ht="30" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2951,60 +3039,60 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E8" s="19">
         <v>46315.5</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="33" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E9" s="20">
         <v>46322.5</v>
@@ -3013,21 +3101,21 @@
         <v>29000</v>
       </c>
       <c r="G9" s="34" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>127</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E10" s="19">
         <v>46322.5</v>
@@ -3036,21 +3124,21 @@
         <v>29000</v>
       </c>
       <c r="G10" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E11" s="20">
         <v>46322.5</v>
@@ -3059,21 +3147,21 @@
         <v>29000</v>
       </c>
       <c r="G11" s="34" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E12" s="19">
         <v>46322.5</v>
@@ -3082,7 +3170,7 @@
         <v>29000</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -3107,28 +3195,30 @@
     <tabColor rgb="FF2A85C5"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="30" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="2" ht="30" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-    </row>
-    <row r="3" ht="18" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="H2"/>
+    </row>
+    <row r="3" ht="18" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
         <v>1</v>
       </c>
@@ -3136,8 +3226,9 @@
       <c r="E3"/>
       <c r="F3"/>
       <c r="G3"/>
-    </row>
-    <row r="5" ht="5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3"/>
+    </row>
+    <row r="5" ht="5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -3145,79 +3236,89 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-    </row>
-    <row r="7" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="4"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>135</v>
-      </c>
       <c r="E7" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B8" s="35">
+        <v>0</v>
+      </c>
+      <c r="C8" s="35">
         <v>5</v>
       </c>
-      <c r="C8" s="12">
+      <c r="D8" s="12">
         <v>144000</v>
-      </c>
-      <c r="D8" s="35">
-        <v>1</v>
       </c>
       <c r="E8" s="35">
         <v>1</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="35">
+        <v>1</v>
+      </c>
+      <c r="G8" s="12">
         <v>4300</v>
       </c>
-      <c r="G8" s="36">
+      <c r="H8" s="36">
         <v>0.2</v>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B9" s="37">
         <f>SUBTOTAL(9,B8:B8)</f>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="37">
         <f>SUBTOTAL(9,C8:C8)</f>
       </c>
-      <c r="D9" s="37">
+      <c r="D9" s="22">
         <f>SUBTOTAL(9,D8:D8)</f>
       </c>
       <c r="E9" s="37">
         <f>SUBTOTAL(9,E8:E8)</f>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="37">
         <f>SUBTOTAL(9,F8:F8)</f>
       </c>
-      <c r="G9" s="21"/>
+      <c r="G9" s="22">
+        <f>SUBTOTAL(9,G8:G8)</f>
+      </c>
+      <c r="H9" s="21"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:G8"/>
+  <autoFilter ref="A7:H8"/>
   <mergeCells count="2">
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="C3:H3"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.2" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -3230,6 +3331,102 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF2A85C5"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="30" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+    </row>
+    <row r="3" ht="18" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+    </row>
+    <row r="5" ht="5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="38" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="A8:G8"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.2" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8&amp;K6B7A86VISITAS GUIADAS</oddHeader>
+    <oddFooter>&amp;L&amp;8Inmobiliaria &amp;&amp; Constructora Vivaldi S.A.C. · RUC 20604145458&amp;R&amp;8Página &amp;P de &amp;N</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF2A85C5"/>
@@ -3251,7 +3448,7 @@
     <row r="1" ht="14" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" ht="30" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -3281,39 +3478,39 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D8" s="11">
         <v>200</v>
@@ -3322,10 +3519,10 @@
         <v>29000</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>13</v>
@@ -3333,13 +3530,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="D9" s="14">
         <v>200</v>
@@ -3348,50 +3545,50 @@
         <v>29000</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="38" t="s">
-        <v>146</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>151</v>
-      </c>
-      <c r="D10" s="39">
+      <c r="A10" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="39" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="D10" s="40">
         <v>200</v>
       </c>
-      <c r="E10" s="40">
+      <c r="E10" s="41">
         <v>29000</v>
       </c>
-      <c r="F10" s="38" t="s">
-        <v>148</v>
-      </c>
-      <c r="G10" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="H10" s="38" t="s">
-        <v>50</v>
+      <c r="F10" s="39" t="s">
+        <v>155</v>
+      </c>
+      <c r="G10" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" s="39" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D11" s="14">
         <v>200</v>
@@ -3400,10 +3597,10 @@
         <v>29000</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>13</v>
@@ -3411,13 +3608,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="D12" s="11">
         <v>200</v>
@@ -3426,10 +3623,10 @@
         <v>29000</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>13</v>
@@ -3437,13 +3634,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D13" s="14">
         <v>200</v>
@@ -3452,10 +3649,10 @@
         <v>29000</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H13" s="13" t="s">
         <v>13</v>
@@ -3463,13 +3660,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D14" s="11">
         <v>200</v>
@@ -3478,10 +3675,10 @@
         <v>29000</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>13</v>
@@ -3489,13 +3686,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="D15" s="14">
         <v>200</v>
@@ -3504,10 +3701,10 @@
         <v>29000</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>13</v>
@@ -3515,13 +3712,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D16" s="11">
         <v>200</v>
@@ -3530,10 +3727,10 @@
         <v>29000</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>13</v>
@@ -3541,13 +3738,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="D17" s="14">
         <v>200</v>
@@ -3556,10 +3753,10 @@
         <v>29000</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>13</v>
@@ -3567,13 +3764,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D18" s="11">
         <v>200</v>
@@ -3582,10 +3779,10 @@
         <v>29000</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>13</v>
@@ -3593,13 +3790,13 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D19" s="14">
         <v>200</v>
@@ -3608,10 +3805,10 @@
         <v>29000</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>13</v>
@@ -3619,13 +3816,13 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="D20" s="11">
         <v>200</v>
@@ -3634,10 +3831,10 @@
         <v>29000</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>13</v>
@@ -3645,13 +3842,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D21" s="14">
         <v>200</v>
@@ -3660,10 +3857,10 @@
         <v>29000</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H21" s="13" t="s">
         <v>13</v>
@@ -3671,13 +3868,13 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D22" s="11">
         <v>200</v>
@@ -3686,10 +3883,10 @@
         <v>29000</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>13</v>
@@ -3697,13 +3894,13 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="D23" s="14">
         <v>200</v>
@@ -3712,10 +3909,10 @@
         <v>29000</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>13</v>
@@ -3723,13 +3920,13 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D24" s="11">
         <v>200</v>
@@ -3738,10 +3935,10 @@
         <v>29000</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>13</v>
@@ -3749,13 +3946,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D25" s="14">
         <v>200</v>
@@ -3764,10 +3961,10 @@
         <v>29000</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H25" s="13" t="s">
         <v>13</v>
@@ -3775,13 +3972,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="D26" s="11">
         <v>200</v>
@@ -3790,10 +3987,10 @@
         <v>29000</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H26" s="10" t="s">
         <v>13</v>
@@ -3801,13 +3998,13 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D27" s="14">
         <v>200</v>
@@ -3816,10 +4013,10 @@
         <v>29000</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H27" s="13" t="s">
         <v>13</v>
@@ -3827,13 +4024,13 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D28" s="11">
         <v>200</v>
@@ -3842,10 +4039,10 @@
         <v>29000</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H28" s="10" t="s">
         <v>13</v>
@@ -3853,13 +4050,13 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B29" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29" s="13" t="s">
         <v>163</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>156</v>
       </c>
       <c r="D29" s="14">
         <v>200</v>
@@ -3868,10 +4065,10 @@
         <v>29000</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H29" s="13" t="s">
         <v>13</v>

</xml_diff>